<commit_message>
Fix UI dark mode styling, improve gas/strom account mapping, enhance cache editor, and remove obsolete Globale Begriffe and Kontenplan sheet
</commit_message>
<xml_diff>
--- a/Systemdaten/TargaListe.xlsx
+++ b/Systemdaten/TargaListe.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fahrzeuge" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fahrzeugtypen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fahrzeuge" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fahrzeugtypen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -682,6 +682,27 @@
       <c r="A23" t="inlineStr">
         <is>
           <t>FN966MX</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>FL060BE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>FW417SB</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>GR426AL</t>
         </is>
       </c>
     </row>

</xml_diff>